<commit_message>
NDVI Sentinel-2 Sep24-May25 integrado - caracterizacion agricola por predio
</commit_message>
<xml_diff>
--- a/outputs/muestra_final.xlsx
+++ b/outputs/muestra_final.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,16 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>observaciones</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ndvi_200m</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>intensidad_agricola</t>
         </is>
       </c>
     </row>
@@ -559,6 +569,14 @@
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>0.342</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -606,6 +624,14 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +679,14 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>0.381</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -700,6 +734,14 @@
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>0.344</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -747,6 +789,14 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -794,6 +844,14 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -841,6 +899,14 @@
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -888,6 +954,14 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -935,6 +1009,14 @@
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -982,6 +1064,14 @@
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>0.383</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1029,6 +1119,14 @@
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1076,6 +1174,14 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1123,6 +1229,14 @@
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
+      <c r="T14" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1170,6 +1284,14 @@
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1217,6 +1339,14 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1264,6 +1394,14 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>0.306</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1311,6 +1449,14 @@
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1358,6 +1504,14 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>0.462</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1405,6 +1559,14 @@
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>0.347</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1452,6 +1614,14 @@
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>0.401</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1499,6 +1669,14 @@
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
+      <c r="T22" t="n">
+        <v>0.368</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1546,6 +1724,14 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
+      <c r="T23" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1593,6 +1779,14 @@
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1640,6 +1834,14 @@
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
+      <c r="T25" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1687,6 +1889,14 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
+      <c r="T26" t="n">
+        <v>0.318</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1734,6 +1944,14 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
+      <c r="T27" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1781,6 +1999,14 @@
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1828,6 +2054,14 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
+      <c r="T29" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1875,6 +2109,14 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
+      <c r="T30" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>media_baja</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1922,6 +2164,14 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
+      <c r="T31" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>media_alta</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
dNDVI estiaje-lluvias integrado - caracterizacion uso suelo por predio
</commit_message>
<xml_diff>
--- a/outputs/muestra_final.xlsx
+++ b/outputs/muestra_final.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,6 +520,16 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>intensidad_agricola</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>dndvi_200m</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>uso_estimado</t>
         </is>
       </c>
     </row>
@@ -577,6 +587,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V2" t="n">
+        <v>0.211</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -632,6 +650,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V3" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -687,6 +713,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V4" t="n">
+        <v>0.229</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -742,6 +776,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V5" t="n">
+        <v>0.251</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -797,6 +839,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V6" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -852,6 +902,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V7" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -907,6 +965,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V8" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -962,6 +1028,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V9" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1017,6 +1091,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V10" t="n">
+        <v>0.224</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1072,6 +1154,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V11" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1127,6 +1217,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V12" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1182,6 +1280,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V13" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1237,6 +1343,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V14" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1292,6 +1406,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V15" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1347,6 +1469,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V16" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1402,6 +1532,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V17" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1457,6 +1595,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V18" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1512,6 +1658,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V19" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1567,6 +1721,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V20" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1622,6 +1784,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V21" t="n">
+        <v>0.215</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1677,6 +1847,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V22" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1732,6 +1910,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V23" t="n">
+        <v>0.218</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1787,6 +1973,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V24" t="n">
+        <v>0.227</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1842,6 +2036,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V25" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1897,6 +2099,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V26" t="n">
+        <v>0.238</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1952,6 +2162,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V27" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>transicion</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2007,6 +2225,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V28" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>cultivo_activo</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2062,6 +2288,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V29" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2117,6 +2351,14 @@
           <t>media_baja</t>
         </is>
       </c>
+      <c r="V30" t="n">
+        <v>0.159</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2172,6 +2414,14 @@
           <t>media_alta</t>
         </is>
       </c>
+      <c r="V31" t="n">
+        <v>0.161</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>cultivo_moderado</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>